<commit_message>
Round 5: second recheck of the flagged rows, rescored
Verified answers from a second model-assisted, human-verified pass on the
five rows flagged in the first scoring: A10 2019-09-23 17:06 (p7, p15),
A31 no (UNSURE), A22 not_stated, A05 not_stated, A08 2020-09-07 04:25
following the earliest-time rule. After rechecking: queue 30/30 (88.6 to
100), unflagged 14/15 (70.2 to 98.8), old model-written labels 15/15 (79.6
to 100), round 4 12/12; A54 is the only difference. The as-submitted
results stay the headline and are unchanged.

The docs say that only rows that disagreed were rechecked, which can only
raise agreement, and that the verifier had already seen the compared values
for A05, A08, A10, and A31. The Pueblo 2103 entry in contradictions.csv is
kept as a possible report error; the audit answer follows the rule.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research/psps_reports/round5/audit_sheet_rechecked.xlsx
+++ b/research/psps_reports/round5/audit_sheet_rechecked.xlsx
@@ -68,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -87,6 +87,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -858,7 +859,7 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>zero</t>
+          <t>not_stated</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -868,7 +869,7 @@
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>PSPS protacol not initiated so not applicable</t>
+          <t>Report says Section 7 is not applicable because PSPS protocols weren't initiated; rules code that as not_stated.</t>
         </is>
       </c>
     </row>
@@ -1017,17 +1018,19 @@
           <t>de-energized; circuit; time</t>
         </is>
       </c>
-      <c r="I9" s="6" t="n">
-        <v>44081.60486111111</v>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>2020-09-07 04:25</t>
+        </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>56</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>Pueblo 2103's 9/7/2020 4:25 (p56) is about 10 hours before every other 9/7 circuit (next: Kanaka 1101 at 14:31, p54). Its Napa neighbor Pueblo 2102 is 9/8/2020 4:07 (p56), so the date is likely an error for 9/8. Treated as an error; the first de-energization is Kanaka 1101 at 14:31.</t>
+          <t>Pueblo 2103 at 9/7 4:25 (p56) is about 10 hours before any other 9/7 circuit and may be a report error, but nothing in the report says so; following the rule.</t>
         </is>
       </c>
     </row>
@@ -1119,15 +1122,19 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>2020/09-25 02:46</t>
+          <t>2019-09-23 17:06</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="n"/>
+          <t>7;15</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Two-phase event; first de-energization Sept 23 at 17:06 (p7). The p4 table's 2020/09-25 02:46 is Bravo phase only, with a year typo.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="86.40000000000001" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1736,12 +1743,12 @@
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>7;8</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>UNSURE: No customers de energized</t>
+          <t>No customers de-energized (p7; Table 1 shows 0 de-energized, p8).</t>
         </is>
       </c>
     </row>
@@ -2200,17 +2207,17 @@
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>not_stated</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>5;10;38</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>UNSURE: No customers de energized</t>
+          <t>UNSURE: no advance notices were sent; shutoff notices went only to the 86 customers de-energized (p38). Leaning no over not_stated.</t>
         </is>
       </c>
     </row>

</xml_diff>